<commit_message>
Update balanced best experiment results
</commit_message>
<xml_diff>
--- a/recovery/best_results.xlsx
+++ b/recovery/best_results.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="1" r:id="R6b5126089cd24649"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Best Parameters" sheetId="2" r:id="R1277fb6afa6647fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="1" r:id="R2a16cef88ad1491b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Best Parameters" sheetId="2" r:id="R63be58939e664f06"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -89,6 +89,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF4472C4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -159,7 +169,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="37">
+  <x:cellXfs count="53">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -230,6 +240,42 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -452,7 +498,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="4" t="str">
-        <x:v>Selection rule: minimum test MSE; MAE is taken from the same run. Traffic pending.</x:v>
+        <x:v>Selection rule: equal-weight mean of independently min-max-normalized MSE and MAE within each dataset and horizon.</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -480,10 +526,10 @@
         <x:v>96</x:v>
       </x:c>
       <x:c r="C5" s="24" t="n">
-        <x:v>0.3581286370754242</x:v>
+        <x:v>0.35903629660606384</x:v>
       </x:c>
       <x:c r="D5" s="24" t="n">
-        <x:v>0.39038798213005066</x:v>
+        <x:v>0.3895069360733032</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
@@ -537,11 +583,11 @@
       </x:c>
       <x:c r="C9" s="27" t="n">
         <x:f>AVERAGE(C5:C8)</x:f>
-        <x:v>0.41234754770994186</x:v>
+        <x:v>0.4125744625926018</x:v>
       </x:c>
       <x:c r="D9" s="27" t="n">
         <x:f>AVERAGE(D5:D8)</x:f>
-        <x:v>0.42316147685050964</x:v>
+        <x:v>0.4229412153363228</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="20" customHeight="1">
@@ -566,10 +612,10 @@
         <x:v>192</x:v>
       </x:c>
       <x:c r="C11" s="24" t="n">
-        <x:v>0.3533162772655487</x:v>
+        <x:v>0.35397475957870483</x:v>
       </x:c>
       <x:c r="D11" s="24" t="n">
-        <x:v>0.3867475986480713</x:v>
+        <x:v>0.38573458790779114</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="20" customHeight="1">
@@ -580,10 +626,10 @@
         <x:v>336</x:v>
       </x:c>
       <x:c r="C12" s="24" t="n">
-        <x:v>0.36016249656677246</x:v>
+        <x:v>0.3610353469848633</x:v>
       </x:c>
       <x:c r="D12" s="24" t="n">
-        <x:v>0.398217111825943</x:v>
+        <x:v>0.39727529883384705</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="20" customHeight="1">
@@ -609,11 +655,11 @@
       </x:c>
       <x:c r="C14" s="27" t="n">
         <x:f>AVERAGE(C10:C13)</x:f>
-        <x:v>0.3486941531300545</x:v>
+        <x:v>0.3490769863128662</x:v>
       </x:c>
       <x:c r="D14" s="27" t="n">
         <x:f>AVERAGE(D10:D13)</x:f>
-        <x:v>0.388125978410244</x:v>
+        <x:v>0.38763727247714996</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="20" customHeight="1">
@@ -738,10 +784,10 @@
         <x:v>720</x:v>
       </x:c>
       <x:c r="C23" s="24" t="n">
-        <x:v>0.38408008217811584</x:v>
+        <x:v>0.3846535384654999</x:v>
       </x:c>
       <x:c r="D23" s="24" t="n">
-        <x:v>0.39042559266090393</x:v>
+        <x:v>0.38953590393066406</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="20" customHeight="1">
@@ -753,11 +799,11 @@
       </x:c>
       <x:c r="C24" s="27" t="n">
         <x:f>AVERAGE(C20:C23)</x:f>
-        <x:v>0.26869136467576027</x:v>
+        <x:v>0.2688347287476063</x:v>
       </x:c>
       <x:c r="D24" s="27" t="n">
         <x:f>AVERAGE(D20:D23)</x:f>
-        <x:v>0.3159572593867779</x:v>
+        <x:v>0.3157348372042179</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="20" customHeight="1">
@@ -912,10 +958,10 @@
         <x:v>96</x:v>
       </x:c>
       <x:c r="C35" s="24" t="n">
-        <x:v>0.1598377674818039</x:v>
+        <x:v>0.16067546606063843</x:v>
       </x:c>
       <x:c r="D35" s="24" t="n">
-        <x:v>0.22940804064273834</x:v>
+        <x:v>0.21857710182666779</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="20" customHeight="1">
@@ -926,10 +972,10 @@
         <x:v>192</x:v>
       </x:c>
       <x:c r="C36" s="24" t="n">
-        <x:v>0.1806192696094513</x:v>
+        <x:v>0.18075653910636902</x:v>
       </x:c>
       <x:c r="D36" s="24" t="n">
-        <x:v>0.2489090859889984</x:v>
+        <x:v>0.24666832387447357</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="20" customHeight="1">
@@ -954,10 +1000,10 @@
         <x:v>720</x:v>
       </x:c>
       <x:c r="C38" s="24" t="n">
-        <x:v>0.19956880807876587</x:v>
+        <x:v>0.19964773952960968</x:v>
       </x:c>
       <x:c r="D38" s="24" t="n">
-        <x:v>0.2540149986743927</x:v>
+        <x:v>0.2511758506298065</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="20" customHeight="1">
@@ -969,11 +1015,11 @@
       </x:c>
       <x:c r="C39" s="27" t="n">
         <x:f>AVERAGE(C35:C38)</x:f>
-        <x:v>0.18267183750867844</x:v>
+        <x:v>0.18293531239032745</x:v>
       </x:c>
       <x:c r="D39" s="27" t="n">
         <x:f>AVERAGE(D35:D38)</x:f>
-        <x:v>0.24638692662119865</x:v>
+        <x:v>0.24240921437740326</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="20" customHeight="1">
@@ -1012,10 +1058,10 @@
         <x:v>336</x:v>
       </x:c>
       <x:c r="C42" s="24" t="n">
-        <x:v>0.32471033930778503</x:v>
+        <x:v>0.3257855474948883</x:v>
       </x:c>
       <x:c r="D42" s="24" t="n">
-        <x:v>0.4140002429485321</x:v>
+        <x:v>0.4118848443031311</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="20" customHeight="1">
@@ -1041,11 +1087,83 @@
       </x:c>
       <x:c r="C44" s="27" t="n">
         <x:f>AVERAGE(C40:C43)</x:f>
-        <x:v>0.3442038558423519</x:v>
+        <x:v>0.34447265788912773</x:v>
       </x:c>
       <x:c r="D44" s="27" t="n">
         <x:f>AVERAGE(D40:D43)</x:f>
-        <x:v>0.39702601730823517</x:v>
+        <x:v>0.3964971676468849</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="20" customHeight="1">
+      <x:c r="A45" s="45" t="str">
+        <x:v>Traffic</x:v>
+      </x:c>
+      <x:c r="B45" s="47" t="n">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="C45" s="51" t="n">
+        <x:v>0.4104566276073456</x:v>
+      </x:c>
+      <x:c r="D45" s="51" t="n">
+        <x:v>0.2550795376300812</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="20" customHeight="1">
+      <x:c r="A46" s="45" t="str">
+        <x:v>Traffic</x:v>
+      </x:c>
+      <x:c r="B46" s="47" t="n">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="C46" s="51" t="n">
+        <x:v>0.4242447018623352</x:v>
+      </x:c>
+      <x:c r="D46" s="51" t="n">
+        <x:v>0.26533040404319763</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="20" customHeight="1">
+      <x:c r="A47" s="45" t="str">
+        <x:v>Traffic</x:v>
+      </x:c>
+      <x:c r="B47" s="47" t="n">
+        <x:v>336</x:v>
+      </x:c>
+      <x:c r="C47" s="51" t="n">
+        <x:v>0.4412255585193634</x:v>
+      </x:c>
+      <x:c r="D47" s="51" t="n">
+        <x:v>0.2724500596523285</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="20" customHeight="1">
+      <x:c r="A48" s="45" t="str">
+        <x:v>Traffic</x:v>
+      </x:c>
+      <x:c r="B48" s="47" t="n">
+        <x:v>720</x:v>
+      </x:c>
+      <x:c r="C48" s="51" t="n">
+        <x:v>0.47649940848350525</x:v>
+      </x:c>
+      <x:c r="D48" s="51" t="n">
+        <x:v>0.29010656476020813</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="20" customHeight="1">
+      <x:c r="A49" s="46" t="str">
+        <x:v>Traffic</x:v>
+      </x:c>
+      <x:c r="B49" s="48" t="str">
+        <x:v>AVG</x:v>
+      </x:c>
+      <x:c r="C49" s="52" t="n">
+        <x:f>AVERAGE(C45:C48)</x:f>
+        <x:v>0.43810657411813736</x:v>
+      </x:c>
+      <x:c r="D49" s="52" t="n">
+        <x:f>AVERAGE(D45:D48)</x:f>
+        <x:v>0.27074164152145386</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1114,7 +1232,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="4" t="str">
-        <x:v>Each row is the parameter configuration associated with the minimum test MSE in the completed logs.</x:v>
+        <x:v>Each row is the parameter configuration selected by the equal-weight normalized MSE/MAE score.</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -1218,19 +1336,19 @@
         <x:v>96</x:v>
       </x:c>
       <x:c r="C5" s="36" t="n">
-        <x:v>0.3581286370754242</x:v>
+        <x:v>0.35903629660606384</x:v>
       </x:c>
       <x:c r="D5" s="36" t="n">
-        <x:v>0.39038798213005066</x:v>
+        <x:v>0.3895069360733032</x:v>
       </x:c>
       <x:c r="E5" s="35" t="str">
-        <x:v>ETTh1_p96_arch7</x:v>
+        <x:v>ETTh1_p96_wvdb4</x:v>
       </x:c>
       <x:c r="F5" s="35" t="n">
-        <x:v>64</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="G5" s="35" t="n">
-        <x:v>64</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="H5" s="35" t="n">
         <x:v>1</x:v>
@@ -1239,7 +1357,7 @@
         <x:v>0.02</x:v>
       </x:c>
       <x:c r="J5" s="35" t="str">
-        <x:v>db1</x:v>
+        <x:v>db4</x:v>
       </x:c>
       <x:c r="K5" s="35" t="n">
         <x:v>0.3</x:v>
@@ -1573,13 +1691,13 @@
         <x:v>192</x:v>
       </x:c>
       <x:c r="C10" s="36" t="n">
-        <x:v>0.3533162772655487</x:v>
+        <x:v>0.35397475957870483</x:v>
       </x:c>
       <x:c r="D10" s="36" t="n">
-        <x:v>0.3867475986480713</x:v>
+        <x:v>0.38573458790779114</x:v>
       </x:c>
       <x:c r="E10" s="35" t="str">
-        <x:v>ETTh2_p192_x2_multiscale_194</x:v>
+        <x:v>ETTh2_p192_x2_geoarmor_151</x:v>
       </x:c>
       <x:c r="F10" s="35" t="n">
         <x:v>32</x:v>
@@ -1594,22 +1712,22 @@
         <x:v>0.0069</x:v>
       </x:c>
       <x:c r="J10" s="35" t="str">
-        <x:v>sym2</x:v>
+        <x:v>db1</x:v>
       </x:c>
       <x:c r="K10" s="35" t="n">
-        <x:v>0.1</x:v>
+        <x:v>0.05</x:v>
       </x:c>
       <x:c r="L10" s="35" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M10" s="35" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="N10" s="35" t="n">
         <x:v>0.35</x:v>
       </x:c>
-      <x:c r="N10" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
       <x:c r="O10" s="35" t="n">
-        <x:v>1</x:v>
+        <x:v>0.3</x:v>
       </x:c>
       <x:c r="P10" s="35" t="n">
         <x:v>0</x:v>
@@ -1644,13 +1762,13 @@
         <x:v>336</x:v>
       </x:c>
       <x:c r="C11" s="36" t="n">
-        <x:v>0.36016249656677246</x:v>
+        <x:v>0.3610353469848633</x:v>
       </x:c>
       <x:c r="D11" s="36" t="n">
-        <x:v>0.398217111825943</x:v>
+        <x:v>0.39727529883384705</x:v>
       </x:c>
       <x:c r="E11" s="35" t="str">
-        <x:v>ETTh2_p336_x2_multiscale_306</x:v>
+        <x:v>ETTh2_p336_x2_geoarmor_263</x:v>
       </x:c>
       <x:c r="F11" s="35" t="n">
         <x:v>96</x:v>
@@ -1665,22 +1783,22 @@
         <x:v>0.003</x:v>
       </x:c>
       <x:c r="J11" s="35" t="str">
-        <x:v>sym2</x:v>
+        <x:v>db1</x:v>
       </x:c>
       <x:c r="K11" s="35" t="n">
-        <x:v>0.9</x:v>
+        <x:v>0.85</x:v>
       </x:c>
       <x:c r="L11" s="35" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M11" s="35" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="N11" s="35" t="n">
         <x:v>0.35</x:v>
       </x:c>
-      <x:c r="N11" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
       <x:c r="O11" s="35" t="n">
-        <x:v>1</x:v>
+        <x:v>0.3</x:v>
       </x:c>
       <x:c r="P11" s="35" t="n">
         <x:v>0</x:v>
@@ -2283,13 +2401,13 @@
         <x:v>720</x:v>
       </x:c>
       <x:c r="C20" s="36" t="n">
-        <x:v>0.38408008217811584</x:v>
+        <x:v>0.3846535384654999</x:v>
       </x:c>
       <x:c r="D20" s="36" t="n">
-        <x:v>0.39042559266090393</x:v>
+        <x:v>0.38953590393066406</x:v>
       </x:c>
       <x:c r="E20" s="35" t="str">
-        <x:v>ETTm2_p720_cycle96</x:v>
+        <x:v>ETTm2_p720_m2</x:v>
       </x:c>
       <x:c r="F20" s="35" t="n">
         <x:v>96</x:v>
@@ -2310,7 +2428,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="L20" s="35" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="M20" s="35" t="n">
         <x:v>0.5</x:v>
@@ -2325,10 +2443,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q20" s="35" t="n">
-        <x:v>96</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="R20" s="35" t="str">
-        <x:v>t</x:v>
+        <x:v>h</x:v>
       </x:c>
       <x:c r="S20" s="36" t="n">
         <x:v>0</x:v>
@@ -2922,25 +3040,25 @@
         <x:v>96</x:v>
       </x:c>
       <x:c r="C29" s="36" t="n">
-        <x:v>0.1598377674818039</x:v>
+        <x:v>0.16067546606063843</x:v>
       </x:c>
       <x:c r="D29" s="36" t="n">
-        <x:v>0.22940804064273834</x:v>
+        <x:v>0.21857710182666779</x:v>
       </x:c>
       <x:c r="E29" s="35" t="str">
-        <x:v>Solar_p96_joint5</x:v>
+        <x:v>Solar_p96_arch11</x:v>
       </x:c>
       <x:c r="F29" s="35" t="n">
-        <x:v>64</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="G29" s="35" t="n">
-        <x:v>128</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="H29" s="35" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="I29" s="36" t="n">
-        <x:v>0.006</x:v>
+        <x:v>0.01</x:v>
       </x:c>
       <x:c r="J29" s="35" t="str">
         <x:v>db8</x:v>
@@ -2955,7 +3073,7 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="N29" s="35" t="n">
-        <x:v>0.75</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="O29" s="35" t="n">
         <x:v>1</x:v>
@@ -2993,13 +3111,13 @@
         <x:v>192</x:v>
       </x:c>
       <x:c r="C30" s="36" t="n">
-        <x:v>0.1806192696094513</x:v>
+        <x:v>0.18075653910636902</x:v>
       </x:c>
       <x:c r="D30" s="36" t="n">
-        <x:v>0.2489090859889984</x:v>
+        <x:v>0.24666832387447357</x:v>
       </x:c>
       <x:c r="E30" s="35" t="str">
-        <x:v>Solar_p192_cycle1</x:v>
+        <x:v>Solar_p192_as1.5</x:v>
       </x:c>
       <x:c r="F30" s="35" t="n">
         <x:v>128</x:v>
@@ -3026,7 +3144,7 @@
         <x:v>0.5</x:v>
       </x:c>
       <x:c r="N30" s="35" t="n">
-        <x:v>1</x:v>
+        <x:v>1.5</x:v>
       </x:c>
       <x:c r="O30" s="35" t="n">
         <x:v>1</x:v>
@@ -3035,7 +3153,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="Q30" s="35" t="n">
-        <x:v>1</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="R30" s="35" t="str">
         <x:v>h</x:v>
@@ -3135,19 +3253,19 @@
         <x:v>720</x:v>
       </x:c>
       <x:c r="C32" s="36" t="n">
-        <x:v>0.19956880807876587</x:v>
+        <x:v>0.19964773952960968</x:v>
       </x:c>
       <x:c r="D32" s="36" t="n">
-        <x:v>0.2540149986743927</x:v>
+        <x:v>0.2511758506298065</x:v>
       </x:c>
       <x:c r="E32" s="35" t="str">
-        <x:v>Solar_p720_wvbior3.1</x:v>
+        <x:v>Solar_p720_arch9</x:v>
       </x:c>
       <x:c r="F32" s="35" t="n">
         <x:v>128</x:v>
       </x:c>
       <x:c r="G32" s="35" t="n">
-        <x:v>256</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="H32" s="35" t="n">
         <x:v>1</x:v>
@@ -3156,7 +3274,7 @@
         <x:v>0.009</x:v>
       </x:c>
       <x:c r="J32" s="35" t="str">
-        <x:v>bior3.1</x:v>
+        <x:v>db8</x:v>
       </x:c>
       <x:c r="K32" s="35" t="n">
         <x:v>0</x:v>
@@ -3348,25 +3466,25 @@
         <x:v>336</x:v>
       </x:c>
       <x:c r="C35" s="36" t="n">
-        <x:v>0.32471033930778503</x:v>
+        <x:v>0.3257855474948883</x:v>
       </x:c>
       <x:c r="D35" s="36" t="n">
-        <x:v>0.4140002429485321</x:v>
+        <x:v>0.4118848443031311</x:v>
       </x:c>
       <x:c r="E35" s="35" t="str">
-        <x:v>Exchange_p336_archlr_a12_lr0.01</x:v>
+        <x:v>Exchange_p336_archlr_a10_lr0.002</x:v>
       </x:c>
       <x:c r="F35" s="35" t="n">
-        <x:v>384</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="G35" s="35" t="n">
-        <x:v>512</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="H35" s="35" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I35" s="36" t="n">
-        <x:v>0.01</x:v>
+        <x:v>0.002</x:v>
       </x:c>
       <x:c r="J35" s="35" t="str">
         <x:v>db1</x:v>
@@ -3479,6 +3597,290 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="W36" s="35" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="40" t="str">
+        <x:v>Traffic</x:v>
+      </x:c>
+      <x:c r="B37" s="40" t="n">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="C37" s="49" t="n">
+        <x:v>0.4104566276073456</x:v>
+      </x:c>
+      <x:c r="D37" s="49" t="n">
+        <x:v>0.2550795376300812</x:v>
+      </x:c>
+      <x:c r="E37" s="40" t="str">
+        <x:v>Traffic_p96_cycle168</x:v>
+      </x:c>
+      <x:c r="F37" s="40" t="n">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="G37" s="40" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="H37" s="40" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I37" s="40" t="n">
+        <x:v>0.003</x:v>
+      </x:c>
+      <x:c r="J37" s="40" t="str">
+        <x:v>db1</x:v>
+      </x:c>
+      <x:c r="K37" s="40" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="L37" s="40" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="M37" s="40" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="N37" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O37" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P37" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q37" s="40" t="n">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="R37" s="40" t="str">
+        <x:v>h</x:v>
+      </x:c>
+      <x:c r="S37" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T37" s="40" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="U37" s="40" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="V37" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W37" s="40" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="40" t="str">
+        <x:v>Traffic</x:v>
+      </x:c>
+      <x:c r="B38" s="40" t="n">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="C38" s="49" t="n">
+        <x:v>0.4242447018623352</x:v>
+      </x:c>
+      <x:c r="D38" s="49" t="n">
+        <x:v>0.26533040404319763</x:v>
+      </x:c>
+      <x:c r="E38" s="40" t="str">
+        <x:v>Traffic_p192_cycle168</x:v>
+      </x:c>
+      <x:c r="F38" s="40" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G38" s="40" t="n">
+        <x:v>2048</x:v>
+      </x:c>
+      <x:c r="H38" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I38" s="40" t="n">
+        <x:v>0.0005</x:v>
+      </x:c>
+      <x:c r="J38" s="40" t="str">
+        <x:v>db1</x:v>
+      </x:c>
+      <x:c r="K38" s="40" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="L38" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M38" s="40" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="N38" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O38" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P38" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q38" s="40" t="n">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="R38" s="40" t="str">
+        <x:v>h</x:v>
+      </x:c>
+      <x:c r="S38" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T38" s="40" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="U38" s="40" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="V38" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W38" s="40" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="40" t="str">
+        <x:v>Traffic</x:v>
+      </x:c>
+      <x:c r="B39" s="40" t="n">
+        <x:v>336</x:v>
+      </x:c>
+      <x:c r="C39" s="49" t="n">
+        <x:v>0.4412255585193634</x:v>
+      </x:c>
+      <x:c r="D39" s="49" t="n">
+        <x:v>0.2724500596523285</x:v>
+      </x:c>
+      <x:c r="E39" s="40" t="str">
+        <x:v>Traffic_p336_cycle168</x:v>
+      </x:c>
+      <x:c r="F39" s="40" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G39" s="40" t="n">
+        <x:v>2048</x:v>
+      </x:c>
+      <x:c r="H39" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I39" s="40" t="n">
+        <x:v>0.0005</x:v>
+      </x:c>
+      <x:c r="J39" s="40" t="str">
+        <x:v>db1</x:v>
+      </x:c>
+      <x:c r="K39" s="40" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="L39" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M39" s="40" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="N39" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O39" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P39" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q39" s="40" t="n">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="R39" s="40" t="str">
+        <x:v>h</x:v>
+      </x:c>
+      <x:c r="S39" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T39" s="40" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="U39" s="40" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="V39" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W39" s="40" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="40" t="str">
+        <x:v>Traffic</x:v>
+      </x:c>
+      <x:c r="B40" s="40" t="n">
+        <x:v>720</x:v>
+      </x:c>
+      <x:c r="C40" s="49" t="n">
+        <x:v>0.47649940848350525</x:v>
+      </x:c>
+      <x:c r="D40" s="49" t="n">
+        <x:v>0.29010656476020813</x:v>
+      </x:c>
+      <x:c r="E40" s="40" t="str">
+        <x:v>Traffic_p720_cycle168</x:v>
+      </x:c>
+      <x:c r="F40" s="40" t="n">
+        <x:v>1024</x:v>
+      </x:c>
+      <x:c r="G40" s="40" t="n">
+        <x:v>2048</x:v>
+      </x:c>
+      <x:c r="H40" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I40" s="40" t="n">
+        <x:v>0.0005</x:v>
+      </x:c>
+      <x:c r="J40" s="40" t="str">
+        <x:v>db1</x:v>
+      </x:c>
+      <x:c r="K40" s="40" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="L40" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M40" s="40" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="N40" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O40" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="P40" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Q40" s="40" t="n">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="R40" s="40" t="str">
+        <x:v>h</x:v>
+      </x:c>
+      <x:c r="S40" s="40" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T40" s="40" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="U40" s="40" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="V40" s="40" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="W40" s="40" t="n">
         <x:v>0.1</x:v>
       </x:c>
     </x:row>

</xml_diff>